<commit_message>
Add Vercel services configuration
</commit_message>
<xml_diff>
--- a/Admin_Data/User_Profiles.xlsx
+++ b/Admin_Data/User_Profiles.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W14"/>
+  <dimension ref="A1:W15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -572,26 +572,26 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>shitt_mann</t>
+          <t>Samarth</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>9087569087</t>
+          <t>9267340578</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>shitt_mann</t>
+          <t>Samarth</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>23</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -615,16 +615,16 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>340000</v>
+        <v>450000</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>business_expansion</t>
+          <t>new_business</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>tailoring</t>
+          <t>food</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -633,16 +633,26 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>700000</v>
+        <v>500000</v>
       </c>
       <c r="O2" t="n">
-        <v>100000</v>
-      </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
+        <v>50000</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>B.Tech CS&amp;E</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Lucknow University</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>600000</v>
+      </c>
       <c r="S2" t="n">
-        <v>300000</v>
+        <v>400000</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -652,170 +662,172 @@
       <c r="U2" t="inlineStr"/>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-09-05 14:07:58</t>
+          <t>2026-09-05 16:32:10</t>
         </is>
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>2026-09-05 14:07:58</t>
+          <t>2026-09-05 16:38:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Sunita Devi</t>
+          <t>shitt_mann</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>9888615763</t>
+          <t>9087569087</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Sunita Devi</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+          <t>shitt_mann</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>male</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Lucknow</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>340000</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>business_expansion</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>tailoring</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>700000</v>
+      </c>
+      <c r="O3" t="n">
+        <v>100000</v>
+      </c>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
+      <c r="S3" t="n">
+        <v>300000</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>2026-09-05 14:07:58</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>2026-09-05 14:07:58</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>damn</t>
+          <t>Sunita Devi</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>9763871067</t>
+          <t>9888615763</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>damn</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>prefer_not</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Uttar Pradesh</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Lucknow</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>450000</v>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>education</t>
-        </is>
-      </c>
+          <t>Sunita Devi</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>B.Con</t>
-        </is>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Lucknow University</t>
-        </is>
-      </c>
-      <c r="R4" t="n">
-        <v>600000</v>
-      </c>
-      <c r="S4" t="n">
-        <v>300000</v>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>2026-09-05 13:38:20</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>2026-09-05 13:38:20</t>
-        </is>
-      </c>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>anb</t>
+          <t>damn</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>9238383287</t>
+          <t>9763871067</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>anb</t>
+          <t>damn</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>19</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>male</t>
+          <t>prefer_not</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -830,38 +842,36 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Kanpur Nagar</t>
+          <t>Lucknow</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>500000</v>
+        <v>450000</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>new_business</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>food</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
-        <v>550000</v>
-      </c>
-      <c r="O5" t="n">
-        <v>150000</v>
-      </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
+          <t>education</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>B.Con</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Lucknow University</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>600000</v>
+      </c>
       <c r="S5" t="n">
-        <v>400000</v>
+        <v>300000</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -871,201 +881,253 @@
       <c r="U5" t="inlineStr"/>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17:02</t>
+          <t>2026-09-05 13:38:20</t>
         </is>
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>2026-09-05 10:17:02</t>
+          <t>2026-09-05 13:38:20</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>fdn</t>
+          <t>anb</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>8263899854</t>
+          <t>9238383287</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>fdn</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+          <t>anb</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>male</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Kanpur Nagar</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>500000</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>new_business</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>550000</v>
+      </c>
+      <c r="O6" t="n">
+        <v>150000</v>
+      </c>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr"/>
+      <c r="S6" t="n">
+        <v>400000</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>2026-09-05 10:17:02</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>2026-09-05 10:17:02</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ahil</t>
+          <t>fdn</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>9876556789</t>
+          <t>8263899854</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Ahil</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>female</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Uttar Pradesh</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>Lucknow</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>230000</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>skill</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>dairy</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="N7" t="n">
-        <v>300000</v>
-      </c>
-      <c r="O7" t="n">
-        <v>100000</v>
-      </c>
+          <t>fdn</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
-      <c r="S7" t="n">
-        <v>200000</v>
-      </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr">
-        <is>
-          <t>2026-09-05 02:41:52</t>
-        </is>
-      </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>2026-09-05 02:42:25</t>
-        </is>
-      </c>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>qwert</t>
+          <t>Ahil</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>9821653467</t>
+          <t>9876556789</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>qwert</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
+          <t>Ahil</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>female</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Lucknow</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>230000</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>skill</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>dairy</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>300000</v>
+      </c>
+      <c r="O8" t="n">
+        <v>100000</v>
+      </c>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
+      <c r="S8" t="n">
+        <v>200000</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr"/>
-      <c r="W8" t="inlineStr"/>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>2026-09-05 02:41:52</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>2026-09-05 02:42:25</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>acvf</t>
+          <t>qwert</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>9872467043</t>
+          <t>9821653467</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>acvf</t>
+          <t>qwert</t>
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -1090,151 +1152,151 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Test User</t>
+          <t>acvf</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>8765676029</t>
+          <t>9872467043</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Test User</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>28</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>male</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Uttar Pradesh</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Lucknow</t>
-        </is>
-      </c>
-      <c r="J10" t="n">
-        <v>240000</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>new_business</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>retail</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
-        <is>
-          <t>new</t>
-        </is>
-      </c>
-      <c r="N10" t="n">
-        <v>200000</v>
-      </c>
-      <c r="O10" t="n">
-        <v>150000</v>
-      </c>
+          <t>acvf</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
-      <c r="S10" t="n">
-        <v>50000</v>
-      </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
-      <c r="V10" t="inlineStr">
-        <is>
-          <t>2026-09-04 18:05:36</t>
-        </is>
-      </c>
-      <c r="W10" t="inlineStr">
-        <is>
-          <t>2026-09-05 03:15:18</t>
-        </is>
-      </c>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>dsj</t>
+          <t>Test User</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>9287398239</t>
+          <t>8765676029</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>dsj</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
+          <t>Test User</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>male</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Lucknow</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>240000</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>new_business</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>retail</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>200000</v>
+      </c>
+      <c r="O11" t="n">
+        <v>150000</v>
+      </c>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
+      <c r="S11" t="n">
+        <v>50000</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="U11" t="inlineStr"/>
-      <c r="V11" t="inlineStr"/>
-      <c r="W11" t="inlineStr"/>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>2026-09-04 18:05:36</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>2026-09-05 03:15:18</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>baca</t>
+          <t>dsj</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>9234567801</t>
+          <t>9287398239</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>baca</t>
+          <t>dsj</t>
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -1259,21 +1321,21 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>abc</t>
+          <t>baca</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>9123456780</t>
+          <t>9234567801</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>abc</t>
+          <t>baca</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -1298,7 +1360,7 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1307,7 +1369,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>9876543210</t>
+          <t>9123456780</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1335,6 +1397,45 @@
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
     </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>9876543210</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>abc</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>